<commit_message>
fix: reconstruct June 30 net worth snapshot from K-line data
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="编辑记录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="持仓表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="净值历史" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="交易流水" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="配置" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="编辑记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="持仓表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="净值历史" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交易流水" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配置" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1107,7 +1107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1189,6 +1189,36 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>收盘记录</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>199516.51</v>
+      </c>
+      <c r="C3" t="n">
+        <v>50781.31</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>250515.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-25430.18250000001</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>收盘记录（回补）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add capital flow tracking (出入金记录)
Track external capital injections/withdrawals with a new modal UI.
Auto-seeds initial capital from cost basis. Shows net capital and
true P&L on the KPI card. New API endpoints /api/capital-flow and
/api/capital-flows. Syncs to GitHub to prevent data loss.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="编辑记录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="持仓表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="净值历史" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="交易流水" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="配置" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="编辑记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="持仓表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="净值历史" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交易流水" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配置" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="出入金" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1497,4 +1498,86 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-01 13:30</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>存入</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>277241.79</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>初始本金（自动记录）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-01 13:30</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>存入</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1088</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>外部资金购入黄金</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: daily P&L deducts capital flows (matches 今日盈亏 KPI)
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="编辑记录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="持仓表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="净值历史" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="交易流水" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="配置" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="出入金" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="编辑记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="持仓表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="净值历史" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交易流水" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配置" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="出入金" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1345,7 +1345,7 @@
         <v>252685.21</v>
       </c>
       <c r="F4" t="n">
-        <v>2169.71</v>
+        <v>1081.71</v>
       </c>
       <c r="G4" t="n">
         <v>-24556.58</v>

</xml_diff>